<commit_message>
exercise 2b and 3a
</commit_message>
<xml_diff>
--- a/Green-Holloway_Ex3A_tables.xlsx
+++ b/Green-Holloway_Ex3A_tables.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patri\W2_Workshop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patri\Documents\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53BAC99B-9EE5-4DC8-9BA5-8CEC4C335738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BD43C9-EC6E-4310-822E-547BCF87A9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22710" yWindow="6870" windowWidth="21045" windowHeight="13290" activeTab="3" xr2:uid="{54D012AC-9917-4171-A189-580612A27BF1}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{54D012AC-9917-4171-A189-580612A27BF1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Events" sheetId="1" r:id="rId1"/>
-    <sheet name="Attendees" sheetId="2" r:id="rId2"/>
-    <sheet name="Registrations" sheetId="3" r:id="rId3"/>
+    <sheet name="Bookings" sheetId="1" r:id="rId1"/>
+    <sheet name="Owners" sheetId="2" r:id="rId2"/>
+    <sheet name="Dogs" sheetId="3" r:id="rId3"/>
     <sheet name="Locations" sheetId="4" r:id="rId4"/>
+    <sheet name="Walks" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>event_name</t>
   </si>
@@ -50,9 +51,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>attendee_id</t>
-  </si>
-  <si>
     <t>first_name</t>
   </si>
   <si>
@@ -65,18 +63,9 @@
     <t>phone</t>
   </si>
   <si>
-    <t xml:space="preserve">event_id </t>
-  </si>
-  <si>
     <t xml:space="preserve">location_id </t>
   </si>
   <si>
-    <t>registration_id</t>
-  </si>
-  <si>
-    <t>event_id</t>
-  </si>
-  <si>
     <t>registration_date</t>
   </si>
   <si>
@@ -95,7 +84,34 @@
     <t>city</t>
   </si>
   <si>
-    <t>state</t>
+    <t>Owner_id</t>
+  </si>
+  <si>
+    <t>Dogs_id</t>
+  </si>
+  <si>
+    <t>owner_id</t>
+  </si>
+  <si>
+    <t>park_name</t>
+  </si>
+  <si>
+    <t>walk_id</t>
+  </si>
+  <si>
+    <t>walk_date</t>
+  </si>
+  <si>
+    <t>duration_minutes</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking_id </t>
+  </si>
+  <si>
+    <t>booking_id</t>
   </si>
 </sst>
 </file>
@@ -500,7 +516,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -509,7 +525,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -534,19 +550,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -560,6 +576,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -567,19 +584,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -596,24 +613,57 @@
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
         <v>17</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F427BEFA-91AC-4FE6-910A-2B0E77035F17}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
       <c r="E1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>